<commit_message>
add second annotation target and format
</commit_message>
<xml_diff>
--- a/annotation_tool/annotation_template.xlsx
+++ b/annotation_tool/annotation_template.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/heste/workspace/sn-caption/annotation_tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831C4AD8-2325-EA40-BFE6-1BAE507E0F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC121F6F-2392-7541-93C6-496A58E39BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5780" yWindow="-28300" windowWidth="33600" windowHeight="13980" activeTab="1" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
+    <workbookView xWindow="-14660" yWindow="-28180" windowWidth="33940" windowHeight="14020" activeTab="1" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
   </bookViews>
   <sheets>
     <sheet name="テンプレート" sheetId="4" r:id="rId1"/>
-    <sheet name="moriy" sheetId="5" r:id="rId2"/>
+    <sheet name="テンプレート_seed10" sheetId="6" r:id="rId2"/>
+    <sheet name="moriy" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="1">moriy!$A$1:$H$101</definedName>
+    <definedName name="_10_denoised_1_tokenized_224p_annotation" localSheetId="1">テンプレート_seed10!$A$1:$H$101</definedName>
+    <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="2">moriy!$A$1:$H$101</definedName>
     <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="0">テンプレート!$A$1:$H$101</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +45,21 @@
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
-  <connection id="1" xr16:uid="{2947C2F0-C812-C44E-8E0B-F2D00BC96894}" name="denoised_1_tokenized_224p_annotation1" type="6" refreshedVersion="8" background="1" saveData="1">
+  <connection id="1" xr16:uid="{DED3BFDE-FE8B-444E-9992-18E390A2A210}" name="10_denoised_1_tokenized_224p_annotation" type="6" refreshedVersion="8" background="1" saveData="1">
+    <textPr codePage="65001" sourceFile="/Users/heste/workspace/sn-caption/data/10_denoised_1_tokenized_224p_annotation.csv" tab="0" comma="1">
+      <textFields count="8">
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+      </textFields>
+    </textPr>
+  </connection>
+  <connection id="2" xr16:uid="{2947C2F0-C812-C44E-8E0B-F2D00BC96894}" name="denoised_1_tokenized_224p_annotation1" type="6" refreshedVersion="8" background="1" saveData="1">
     <textPr codePage="65001" sourceFile="/Users/heste/workspace/sn-caption/data/denoised_1_tokenized_224p_annotation.csv" tab="0" comma="1">
       <textFields count="8">
         <textField/>
@@ -56,7 +73,7 @@
       </textFields>
     </textPr>
   </connection>
-  <connection id="2" xr16:uid="{6CA83349-B20A-414D-BA20-B259599B563B}" name="denoised_1_tokenized_224p_annotation11" type="6" refreshedVersion="8" background="1" saveData="1">
+  <connection id="3" xr16:uid="{6CA83349-B20A-414D-BA20-B259599B563B}" name="denoised_1_tokenized_224p_annotation11" type="6" refreshedVersion="8" background="1" saveData="1">
     <textPr codePage="65001" sourceFile="/Users/heste/workspace/sn-caption/data/denoised_1_tokenized_224p_annotation.csv" tab="0" comma="1">
       <textFields count="8">
         <textField/>
@@ -74,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="428">
   <si>
     <t>id</t>
   </si>
@@ -1043,6 +1060,382 @@
       <t xml:space="preserve">カンソウ </t>
     </rPh>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>実況者はwouldのつもりでwillって言ってそう（口語表現？）</t>
+    <rPh sb="0" eb="2">
+      <t xml:space="preserve">ジッキョウｓｈ </t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t xml:space="preserve">シャ </t>
+    </rPh>
+    <rPh sb="20" eb="21">
+      <t xml:space="preserve">イッテソウ </t>
+    </rPh>
+    <rPh sb="26" eb="30">
+      <t xml:space="preserve">コウゴヒョウゲン </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2 3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>he 困る</t>
+    <rPh sb="3" eb="4">
+      <t xml:space="preserve">コマル </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>And the Argentine is enjoying quite a renaissance at the moment.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>迷った。2ぽいかも</t>
+    <rPh sb="0" eb="1">
+      <t xml:space="preserve">マヨッタ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gignac arrives and Gignac scores!</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>spy =&gt; spike?</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Petrushan has to score again.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>付加的情報混じりの感想</t>
+    <rPh sb="0" eb="5">
+      <t xml:space="preserve">フカテキジョウホウ </t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t xml:space="preserve">マジリノカンソウ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>迷</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1と迷った</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>罵倒の意を込めた比喩表現</t>
+    <rPh sb="0" eb="2">
+      <t xml:space="preserve">バトウ </t>
+    </rPh>
+    <rPh sb="8" eb="12">
+      <t xml:space="preserve">ヒユヒョウゲン </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ちょいノイズ？</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Now a idea.</t>
+  </si>
+  <si>
+    <t>He's smart because he's a fake.</t>
+  </si>
+  <si>
+    <t>It's Alaba and Alonso at the heart of that by in defence so it is very much unfamiliar looking defensive line for the home side.</t>
+  </si>
+  <si>
+    <t>When we say holding in the box, we're not talking about a foul now.</t>
+  </si>
+  <si>
+    <t>2015-02-15 - 14-30 AC Milan 1 - 1 Empoli</t>
+  </si>
+  <si>
+    <t>...Menes really is the... ...inspiration for Milan... ...at the moment.</t>
+  </si>
+  <si>
+    <t>Dani Alves is trying to score.</t>
+  </si>
+  <si>
+    <t>Alexander has a problem with the ball.</t>
+  </si>
+  <si>
+    <t>He became much coveted after his time at Southampton, which began here.</t>
+  </si>
+  <si>
+    <t>Mkhmedi.</t>
+  </si>
+  <si>
+    <t>The number 19 Ivan Cavallero.</t>
+  </si>
+  <si>
+    <t>Ronaldo got a hat-trick that day as I mentioned.</t>
+  </si>
+  <si>
+    <t>Marcelo wanted to leave first for Kroos, he gives it directly to the rival.</t>
+  </si>
+  <si>
+    <t>Now the counter-attack.</t>
+  </si>
+  <si>
+    <t>He's been controlling all these things.</t>
+  </si>
+  <si>
+    <t>Kjezo again.</t>
+  </si>
+  <si>
+    <t>Paderborn from the beginning with a clear defense concept.</t>
+  </si>
+  <si>
+    <t>Koke.</t>
+  </si>
+  <si>
+    <t>He shot from a distance.</t>
+  </si>
+  <si>
+    <t>The problem for FC Barcelona is Alventosa's presence.</t>
+  </si>
+  <si>
+    <t>Calcio is returning, which, I think, all fans of the series are very happy about.</t>
+  </si>
+  <si>
+    <t>Hey!</t>
+  </si>
+  <si>
+    <t>Hasn't yet been a break in play.</t>
+  </si>
+  <si>
+    <t>Dani Alves is playing with a traditional Juventus' style.</t>
+  </si>
+  <si>
+    <t>I don't think so.</t>
+  </si>
+  <si>
+    <t>The Zinedine Zidane team are trying to get the ball out, Toni Kroos is looking for it, it's a bad pass.</t>
+  </si>
+  <si>
+    <t>Now Hulk up.</t>
+  </si>
+  <si>
+    <t>And then the non-rule climbing handball.</t>
+  </si>
+  <si>
+    <t>Vidal.</t>
+  </si>
+  <si>
+    <t>Does the little pass inside.</t>
+  </si>
+  <si>
+    <t>Depor will come out obviously looking to defend their goal especially over the first 20 minutes or so.</t>
+  </si>
+  <si>
+    <t>There was no flag.</t>
+  </si>
+  <si>
+    <t>Chelsea in those wide areas.</t>
+  </si>
+  <si>
+    <t>Everything you can win by 1-0 is always very dangerous.</t>
+  </si>
+  <si>
+    <t>The player of the German national team scores the first Juventus ball in the new season.</t>
+  </si>
+  <si>
+    <t>So good start here for the Galicians.</t>
+  </si>
+  <si>
+    <t>Rakitic.</t>
+  </si>
+  <si>
+    <t>Another long ball.</t>
+  </si>
+  <si>
+    <t>Mario Götze is left to Stefan Ilsenker.</t>
+  </si>
+  <si>
+    <t>Nacho outside to the Brazilian left back.</t>
+  </si>
+  <si>
+    <t>Good wall from Bernardeschi.</t>
+  </si>
+  <si>
+    <t>Shaquille has failed.</t>
+  </si>
+  <si>
+    <t>Burak is turning.</t>
+  </si>
+  <si>
+    <t>He scored a yellow-red goal in Lviv.</t>
+  </si>
+  <si>
+    <t>Ribéry, quickly with Lewandowski.</t>
+  </si>
+  <si>
+    <t>He shoots the header.</t>
+  </si>
+  <si>
+    <t>I think he's capable of it.</t>
+  </si>
+  <si>
+    <t>That's why the great good of European football covered his signature.</t>
+  </si>
+  <si>
+    <t>Trapp!</t>
+  </si>
+  <si>
+    <t>But I think everybody knew Cristiano Ronaldo was going to go for goal from that position.</t>
+  </si>
+  <si>
+    <t>It's going to move.</t>
+  </si>
+  <si>
+    <t>And got themselves right back in the game.</t>
+  </si>
+  <si>
+    <t>Although it's just going to beat Marquinhos.</t>
+  </si>
+  <si>
+    <t>Chalhanoglu helps it on towards Kiesling.</t>
+  </si>
+  <si>
+    <t>I must say that they are taking advantage of the change of rules.</t>
+  </si>
+  <si>
+    <t>This is not good for PSG.</t>
+  </si>
+  <si>
+    <t>The ball continues to be on the left side.</t>
+  </si>
+  <si>
+    <t>Hilbert under pressure from Costa.</t>
+  </si>
+  <si>
+    <t>Ventus again.</t>
+  </si>
+  <si>
+    <t>Intuitive Marcelo, that opening by Fran Beltran, made Kevin doubt just enough so that no one touched the ball.</t>
+  </si>
+  <si>
+    <t>Meha is actually the right one on the ball.</t>
+  </si>
+  <si>
+    <t>In a practically full Camp Nou.</t>
+  </si>
+  <si>
+    <t>They say he was on the list of Aurelio de Laurentiis, the president of Naples, after the sale of Gonçalo Higuain.</t>
+  </si>
+  <si>
+    <t>Penalty shout at both ends.</t>
+  </si>
+  <si>
+    <t>It's a very tight ball.</t>
+  </si>
+  <si>
+    <t>You have to say Arsenal have done well with that.</t>
+  </si>
+  <si>
+    <t>Lobotka.</t>
+  </si>
+  <si>
+    <t>First from Kacunga and last from Lukas Rupp.</t>
+  </si>
+  <si>
+    <t>Laura now in possession looking for a free kick that doesn't come.</t>
+  </si>
+  <si>
+    <t>Lowry lost track of it.</t>
+  </si>
+  <si>
+    <t>Vermaelen for Macerano.</t>
+  </si>
+  <si>
+    <t>They were incredible.</t>
+  </si>
+  <si>
+    <t>Teams that will consider those positions to be the minimum of their domestic requirements for this season again.</t>
+  </si>
+  <si>
+    <t>It was not his natural position, but he had many casualties in that demarcation.</t>
+  </si>
+  <si>
+    <t>And now the card is being shown.</t>
+  </si>
+  <si>
+    <t>Isco, little flick to the back post.</t>
+  </si>
+  <si>
+    <t>Because there are many people who want to buy an Italian star.</t>
+  </si>
+  <si>
+    <t>I think I have the statistics, and Ivanovic has scored 27 goals since August 2010.</t>
+  </si>
+  <si>
+    <t>I think he trusts a lot that he will have space and that he can kill him on the counter.</t>
+  </si>
+  <si>
+    <t>I think he's a good player, Adam Lallana.</t>
+  </si>
+  <si>
+    <t>And he gives them stability in the heart of the midfield.</t>
+  </si>
+  <si>
+    <t>Burak.</t>
+  </si>
+  <si>
+    <t>Maybe they changed their mind.</t>
+  </si>
+  <si>
+    <t>You can whistle a foul, you can not whistle a foul and therefore the VAR does not enter there.</t>
+  </si>
+  <si>
+    <t>Cristiano Ronaldo's goal is repeated.</t>
+  </si>
+  <si>
+    <t>Sergi Roberto getting ready for a shot.</t>
+  </si>
+  <si>
+    <t>Aspire Cueta.</t>
+  </si>
+  <si>
+    <t>Keline.</t>
+  </si>
+  <si>
+    <t>This is what we are saying.</t>
+  </si>
+  <si>
+    <t>This is a very powerful football game that the team of André Breitenreiter offers in this early phase, but they are set for it.</t>
+  </si>
+  <si>
+    <t>Atletico Madrid scored the twelfth goal.</t>
+  </si>
+  <si>
+    <t>And he didn't just know, he scored a perfect goal.</t>
+  </si>
+  <si>
+    <t>On Cruz brings him down it'll be another free kick they'll have to be taken a few meters back.</t>
+  </si>
+  <si>
+    <t>It's a failed interception, Ronaldo has Benzema inside, can't get around Lopo.</t>
+  </si>
+  <si>
+    <t>All attacks are thrown in by the Spanish ex-world champion.</t>
+  </si>
+  <si>
+    <t>The pitch is strangely in poor condition normally early on in the season.</t>
+  </si>
+  <si>
+    <t>He saves the ball.</t>
+  </si>
+  <si>
+    <t>Cristiano Ronaldo.</t>
   </si>
 </sst>
 </file>
@@ -1094,7 +1487,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1112,6 +1505,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1131,11 +1530,15 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="denoised_1_tokenized_224p_annotation" connectionId="1" xr16:uid="{635E7587-0BD4-7441-80A8-1B051F2B3EE9}" autoFormatId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="denoised_1_tokenized_224p_annotation" connectionId="2" xr16:uid="{635E7587-0BD4-7441-80A8-1B051F2B3EE9}" autoFormatId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="denoised_1_tokenized_224p_annotation" connectionId="2" xr16:uid="{28FAE329-83B7-BB4C-97D0-3BAFBE2A19B7}" autoFormatId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="10_denoised_1_tokenized_224p_annotation" connectionId="1" xr16:uid="{4A66B805-C96D-3D4B-90B1-DD78F95E1CDE}" autoFormatId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="denoised_1_tokenized_224p_annotation" connectionId="3" xr16:uid="{28FAE329-83B7-BB4C-97D0-3BAFBE2A19B7}" autoFormatId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3187,6 +3590,1755 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF2E0F6F-CB5F-E946-BB3D-A6719BC75C1A}">
+  <dimension ref="A1:H101"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="80.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="21">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="21">
+      <c r="A2">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="7">
+        <v>0.16597222222222222</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0.17222222222222225</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="21">
+      <c r="A3">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7">
+        <v>0.24583333333333335</v>
+      </c>
+      <c r="D3" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="21">
+      <c r="A4">
+        <v>318</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="7">
+        <v>1.8749999999999999E-2</v>
+      </c>
+      <c r="D4" s="7">
+        <v>2.7083333333333334E-2</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="21">
+      <c r="A5">
+        <v>341</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="7">
+        <v>8.2638888888888887E-2</v>
+      </c>
+      <c r="D5" s="7">
+        <v>8.7500000000000008E-2</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="21">
+      <c r="A6">
+        <v>394</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="D6" s="7">
+        <v>0.21319444444444444</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="21">
+      <c r="A7">
+        <v>414</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0.28472222222222221</v>
+      </c>
+      <c r="D7" s="7">
+        <v>0.29097222222222224</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="21">
+      <c r="A8">
+        <v>422</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0.31041666666666667</v>
+      </c>
+      <c r="D8" s="7">
+        <v>0.31666666666666665</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="21">
+      <c r="A9">
+        <v>437</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="7">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D9" s="7">
+        <v>0.35486111111111113</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="21">
+      <c r="A10">
+        <v>491</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="7">
+        <v>0.50069444444444444</v>
+      </c>
+      <c r="D10" s="7">
+        <v>0.51111111111111118</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="21">
+      <c r="A11">
+        <v>502</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="7">
+        <v>0.52777777777777779</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.53055555555555556</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="21">
+      <c r="A12">
+        <v>529</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="7">
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="D12" s="7">
+        <v>0.64930555555555558</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="21">
+      <c r="A13">
+        <v>607</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="7">
+        <v>0.8652777777777777</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.86875000000000002</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="21">
+      <c r="A14">
+        <v>636</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="7">
+        <v>0.92361111111111116</v>
+      </c>
+      <c r="D14" s="7">
+        <v>0.9277777777777777</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="21">
+      <c r="A15">
+        <v>655</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="7">
+        <v>0.97361111111111109</v>
+      </c>
+      <c r="D15" s="7">
+        <v>0.9868055555555556</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="21">
+      <c r="A16">
+        <v>674</v>
+      </c>
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="6">
+        <v>1.0326388888888889</v>
+      </c>
+      <c r="D16" s="6">
+        <v>1.0395833333333333</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="21">
+      <c r="A17">
+        <v>707</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="6">
+        <v>1.1847222222222222</v>
+      </c>
+      <c r="D17" s="6">
+        <v>1.1937499999999999</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="21">
+      <c r="A18">
+        <v>760</v>
+      </c>
+      <c r="B18" t="s">
+        <v>334</v>
+      </c>
+      <c r="C18" s="7">
+        <v>0.72777777777777775</v>
+      </c>
+      <c r="D18" s="7">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="21">
+      <c r="A19">
+        <v>778</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="7">
+        <v>4.7916666666666663E-2</v>
+      </c>
+      <c r="D19" s="7">
+        <v>5.2777777777777778E-2</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="42">
+      <c r="A20">
+        <v>885</v>
+      </c>
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="7">
+        <v>0.7583333333333333</v>
+      </c>
+      <c r="D20" s="7">
+        <v>0.77013888888888893</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="21">
+      <c r="A21">
+        <v>890</v>
+      </c>
+      <c r="B21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="7">
+        <v>0.78263888888888899</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.79236111111111107</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="21">
+      <c r="A22">
+        <v>953</v>
+      </c>
+      <c r="B22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="6">
+        <v>1.6520833333333333</v>
+      </c>
+      <c r="D22" s="6">
+        <v>1.6569444444444443</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="21">
+      <c r="A23">
+        <v>955</v>
+      </c>
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="6">
+        <v>1.6604166666666667</v>
+      </c>
+      <c r="D23" s="6">
+        <v>1.6659722222222222</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="21">
+      <c r="A24">
+        <v>960</v>
+      </c>
+      <c r="B24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="6">
+        <v>1.6729166666666666</v>
+      </c>
+      <c r="D24" s="6">
+        <v>1.6763888888888889</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="21">
+      <c r="A25">
+        <v>961</v>
+      </c>
+      <c r="B25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1.675</v>
+      </c>
+      <c r="D25" s="6">
+        <v>1.6777777777777778</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="21">
+      <c r="A26">
+        <v>998</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="6">
+        <v>1.8381944444444445</v>
+      </c>
+      <c r="D26" s="6">
+        <v>1.8472222222222223</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="21">
+      <c r="A27">
+        <v>1029</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" s="7">
+        <v>7.5694444444444439E-2</v>
+      </c>
+      <c r="D27" s="7">
+        <v>8.1250000000000003E-2</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="21">
+      <c r="A28">
+        <v>1067</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" s="7">
+        <v>0.21805555555555556</v>
+      </c>
+      <c r="D28" s="7">
+        <v>0.22083333333333333</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="21">
+      <c r="A29">
+        <v>1207</v>
+      </c>
+      <c r="B29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" s="7">
+        <v>0.58819444444444446</v>
+      </c>
+      <c r="D29" s="7">
+        <v>0.59166666666666667</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="21">
+      <c r="A30">
+        <v>1318</v>
+      </c>
+      <c r="B30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="6">
+        <v>1.0090277777777776</v>
+      </c>
+      <c r="D30" s="6">
+        <v>1.0111111111111111</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="21">
+      <c r="A31">
+        <v>1542</v>
+      </c>
+      <c r="B31" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="6">
+        <v>1.6416666666666666</v>
+      </c>
+      <c r="D31" s="6">
+        <v>1.6458333333333333</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="21">
+      <c r="A32">
+        <v>1616</v>
+      </c>
+      <c r="B32" t="s">
+        <v>5</v>
+      </c>
+      <c r="C32" s="6">
+        <v>1.8243055555555554</v>
+      </c>
+      <c r="D32" s="6">
+        <v>1.8263888888888891</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="21">
+      <c r="A33">
+        <v>1636</v>
+      </c>
+      <c r="B33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33" s="6">
+        <v>1.8694444444444445</v>
+      </c>
+      <c r="D33" s="6">
+        <v>1.8729166666666668</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="21">
+      <c r="A34">
+        <v>1661</v>
+      </c>
+      <c r="B34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="7">
+        <v>0.11527777777777777</v>
+      </c>
+      <c r="D34" s="7">
+        <v>0.11875000000000001</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="21">
+      <c r="A35">
+        <v>1710</v>
+      </c>
+      <c r="B35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C35" s="7">
+        <v>0.32083333333333336</v>
+      </c>
+      <c r="D35" s="7">
+        <v>0.32708333333333334</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="21">
+      <c r="A36">
+        <v>1716</v>
+      </c>
+      <c r="B36" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="7">
+        <v>0.33819444444444446</v>
+      </c>
+      <c r="D36" s="7">
+        <v>0.34375</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="21">
+      <c r="A37">
+        <v>1725</v>
+      </c>
+      <c r="B37" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" s="7">
+        <v>0.38125000000000003</v>
+      </c>
+      <c r="D37" s="7">
+        <v>0.38680555555555557</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="21">
+      <c r="A38">
+        <v>1948</v>
+      </c>
+      <c r="B38" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38" s="6">
+        <v>1.3451388888888889</v>
+      </c>
+      <c r="D38" s="6">
+        <v>1.3472222222222223</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="21">
+      <c r="A39">
+        <v>2125</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" s="7">
+        <v>0.14444444444444446</v>
+      </c>
+      <c r="D39" s="7">
+        <v>0.14583333333333334</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="21">
+      <c r="A40">
+        <v>2130</v>
+      </c>
+      <c r="B40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" s="7">
+        <v>0.15347222222222223</v>
+      </c>
+      <c r="D40" s="7">
+        <v>0.15694444444444444</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="21">
+      <c r="A41">
+        <v>2327</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="6">
+        <v>1.4104166666666667</v>
+      </c>
+      <c r="D41" s="6">
+        <v>1.4118055555555555</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="21">
+      <c r="A42">
+        <v>2362</v>
+      </c>
+      <c r="B42" t="s">
+        <v>8</v>
+      </c>
+      <c r="C42" s="6">
+        <v>1.4916666666666665</v>
+      </c>
+      <c r="D42" s="6">
+        <v>1.4958333333333333</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="21">
+      <c r="A43">
+        <v>2387</v>
+      </c>
+      <c r="B43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="6">
+        <v>1.5881944444444445</v>
+      </c>
+      <c r="D43" s="6">
+        <v>1.5895833333333333</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="42">
+      <c r="A44">
+        <v>2489</v>
+      </c>
+      <c r="B44" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="7">
+        <v>0.1986111111111111</v>
+      </c>
+      <c r="D44" s="7">
+        <v>0.21319444444444444</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="21">
+      <c r="A45">
+        <v>2507</v>
+      </c>
+      <c r="B45" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="7">
+        <v>0.26597222222222222</v>
+      </c>
+      <c r="D45" s="7">
+        <v>0.2722222222222222</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="21">
+      <c r="A46">
+        <v>2587</v>
+      </c>
+      <c r="B46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="7">
+        <v>0.59930555555555554</v>
+      </c>
+      <c r="D46" s="7">
+        <v>0.6069444444444444</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="21">
+      <c r="A47">
+        <v>2594</v>
+      </c>
+      <c r="B47" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="7">
+        <v>0.61319444444444449</v>
+      </c>
+      <c r="D47" s="7">
+        <v>0.62777777777777777</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="21">
+      <c r="A48">
+        <v>2674</v>
+      </c>
+      <c r="B48" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" s="7">
+        <v>0.84791666666666676</v>
+      </c>
+      <c r="D48" s="7">
+        <v>0.86944444444444446</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="21">
+      <c r="A49">
+        <v>2687</v>
+      </c>
+      <c r="B49" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" s="7">
+        <v>0.8979166666666667</v>
+      </c>
+      <c r="D49" s="7">
+        <v>0.91249999999999998</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="21">
+      <c r="A50">
+        <v>2837</v>
+      </c>
+      <c r="B50" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" s="6">
+        <v>1.4749999999999999</v>
+      </c>
+      <c r="D50" s="6">
+        <v>1.4861111111111109</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="21">
+      <c r="A51">
+        <v>2916</v>
+      </c>
+      <c r="B51" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51" s="6">
+        <v>1.6256944444444443</v>
+      </c>
+      <c r="D51" s="6">
+        <v>1.6465277777777778</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="42">
+      <c r="A52">
+        <v>2938</v>
+      </c>
+      <c r="B52" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" s="6">
+        <v>1.7055555555555555</v>
+      </c>
+      <c r="D52" s="6">
+        <v>1.7138888888888888</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="21">
+      <c r="A53">
+        <v>2990</v>
+      </c>
+      <c r="B53" t="s">
+        <v>6</v>
+      </c>
+      <c r="C53" s="7">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="D53" s="7">
+        <v>5.8333333333333327E-2</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="21">
+      <c r="A54">
+        <v>3121</v>
+      </c>
+      <c r="B54" t="s">
+        <v>6</v>
+      </c>
+      <c r="C54" s="7">
+        <v>0.34861111111111115</v>
+      </c>
+      <c r="D54" s="7">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="21">
+      <c r="A55">
+        <v>3201</v>
+      </c>
+      <c r="B55" t="s">
+        <v>6</v>
+      </c>
+      <c r="C55" s="7">
+        <v>0.47013888888888888</v>
+      </c>
+      <c r="D55" s="7">
+        <v>0.47500000000000003</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="21">
+      <c r="A56">
+        <v>3241</v>
+      </c>
+      <c r="B56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C56" s="7">
+        <v>0.53194444444444444</v>
+      </c>
+      <c r="D56" s="7">
+        <v>0.53333333333333333</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="21">
+      <c r="A57">
+        <v>3311</v>
+      </c>
+      <c r="B57" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="6">
+        <v>1.3645833333333333</v>
+      </c>
+      <c r="D57" s="6">
+        <v>1.3673611111111112</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="21">
+      <c r="A58">
+        <v>3428</v>
+      </c>
+      <c r="B58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" s="6">
+        <v>1.6319444444444444</v>
+      </c>
+      <c r="D58" s="6">
+        <v>1.6354166666666667</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="21">
+      <c r="A59">
+        <v>3459</v>
+      </c>
+      <c r="B59" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" s="6">
+        <v>1.7097222222222221</v>
+      </c>
+      <c r="D59" s="6">
+        <v>1.7145833333333333</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="21">
+      <c r="A60">
+        <v>3468</v>
+      </c>
+      <c r="B60" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" s="6">
+        <v>1.7249999999999999</v>
+      </c>
+      <c r="D60" s="6">
+        <v>1.7277777777777779</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="21">
+      <c r="A61">
+        <v>3485</v>
+      </c>
+      <c r="B61" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" s="6">
+        <v>1.7583333333333335</v>
+      </c>
+      <c r="D61" s="6">
+        <v>1.7618055555555554</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="21">
+      <c r="A62">
+        <v>3616</v>
+      </c>
+      <c r="B62" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="7">
+        <v>0.24444444444444446</v>
+      </c>
+      <c r="D62" s="7">
+        <v>0.24652777777777779</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="21">
+      <c r="A63">
+        <v>3664</v>
+      </c>
+      <c r="B63" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" s="7">
+        <v>0.34791666666666665</v>
+      </c>
+      <c r="D63" s="7">
+        <v>0.3520833333333333</v>
+      </c>
+      <c r="E63" s="5" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="21">
+      <c r="A64">
+        <v>3738</v>
+      </c>
+      <c r="B64" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" s="7">
+        <v>0.4993055555555555</v>
+      </c>
+      <c r="D64" s="7">
+        <v>0.50138888888888888</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="21">
+      <c r="A65">
+        <v>3894</v>
+      </c>
+      <c r="B65" t="s">
+        <v>7</v>
+      </c>
+      <c r="C65" s="7">
+        <v>0.9243055555555556</v>
+      </c>
+      <c r="D65" s="7">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="21">
+      <c r="A66">
+        <v>3921</v>
+      </c>
+      <c r="B66" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" s="7">
+        <v>0.99097222222222225</v>
+      </c>
+      <c r="D66" s="7">
+        <v>0.99375000000000002</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="21">
+      <c r="A67">
+        <v>3940</v>
+      </c>
+      <c r="B67" t="s">
+        <v>7</v>
+      </c>
+      <c r="C67" s="6">
+        <v>1.0381944444444444</v>
+      </c>
+      <c r="D67" s="6">
+        <v>1.0430555555555556</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="21">
+      <c r="A68">
+        <v>3990</v>
+      </c>
+      <c r="B68" t="s">
+        <v>7</v>
+      </c>
+      <c r="C68" s="6">
+        <v>1.1708333333333334</v>
+      </c>
+      <c r="D68" s="6">
+        <v>1.1736111111111112</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="21">
+      <c r="A69">
+        <v>4261</v>
+      </c>
+      <c r="B69" t="s">
+        <v>18</v>
+      </c>
+      <c r="C69" s="7">
+        <v>7.013888888888889E-2</v>
+      </c>
+      <c r="D69" s="7">
+        <v>7.9166666666666663E-2</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="21">
+      <c r="A70">
+        <v>4400</v>
+      </c>
+      <c r="B70" t="s">
+        <v>18</v>
+      </c>
+      <c r="C70" s="7">
+        <v>0.56111111111111112</v>
+      </c>
+      <c r="D70" s="7">
+        <v>0.56319444444444444</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="21">
+      <c r="A71">
+        <v>4432</v>
+      </c>
+      <c r="B71" t="s">
+        <v>18</v>
+      </c>
+      <c r="C71" s="7">
+        <v>0.64722222222222225</v>
+      </c>
+      <c r="D71" s="7">
+        <v>0.65555555555555556</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="21">
+      <c r="A72">
+        <v>4440</v>
+      </c>
+      <c r="B72" t="s">
+        <v>18</v>
+      </c>
+      <c r="C72" s="7">
+        <v>0.66527777777777775</v>
+      </c>
+      <c r="D72" s="7">
+        <v>0.66875000000000007</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="21">
+      <c r="A73">
+        <v>4565</v>
+      </c>
+      <c r="B73" t="s">
+        <v>18</v>
+      </c>
+      <c r="C73" s="6">
+        <v>1.0743055555555556</v>
+      </c>
+      <c r="D73" s="6">
+        <v>1.0777777777777777</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="21">
+      <c r="A74">
+        <v>4796</v>
+      </c>
+      <c r="B74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C74" s="6">
+        <v>1.8625</v>
+      </c>
+      <c r="D74" s="6">
+        <v>1.8694444444444445</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="21">
+      <c r="A75">
+        <v>4848</v>
+      </c>
+      <c r="B75" t="s">
+        <v>14</v>
+      </c>
+      <c r="C75" s="7">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="D75" s="7">
+        <v>5.8333333333333327E-2</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="21">
+      <c r="A76">
+        <v>4855</v>
+      </c>
+      <c r="B76" t="s">
+        <v>14</v>
+      </c>
+      <c r="C76" s="7">
+        <v>7.0833333333333331E-2</v>
+      </c>
+      <c r="D76" s="7">
+        <v>7.7083333333333337E-2</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="21">
+      <c r="A77">
+        <v>4909</v>
+      </c>
+      <c r="B77" t="s">
+        <v>14</v>
+      </c>
+      <c r="C77" s="7">
+        <v>0.20138888888888887</v>
+      </c>
+      <c r="D77" s="7">
+        <v>0.20486111111111113</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="21">
+      <c r="A78">
+        <v>5004</v>
+      </c>
+      <c r="B78" t="s">
+        <v>14</v>
+      </c>
+      <c r="C78" s="7">
+        <v>0.50555555555555554</v>
+      </c>
+      <c r="D78" s="7">
+        <v>0.51388888888888895</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="21">
+      <c r="A79">
+        <v>5058</v>
+      </c>
+      <c r="B79" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79" s="7">
+        <v>0.66388888888888886</v>
+      </c>
+      <c r="D79" s="7">
+        <v>0.66805555555555562</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="21">
+      <c r="A80">
+        <v>5077</v>
+      </c>
+      <c r="B80" t="s">
+        <v>14</v>
+      </c>
+      <c r="C80" s="7">
+        <v>0.71527777777777779</v>
+      </c>
+      <c r="D80" s="7">
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="21">
+      <c r="A81">
+        <v>5127</v>
+      </c>
+      <c r="B81" t="s">
+        <v>14</v>
+      </c>
+      <c r="C81" s="7">
+        <v>0.9458333333333333</v>
+      </c>
+      <c r="D81" s="7">
+        <v>0.96250000000000002</v>
+      </c>
+      <c r="E81" s="5" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="21">
+      <c r="A82">
+        <v>5149</v>
+      </c>
+      <c r="B82" t="s">
+        <v>14</v>
+      </c>
+      <c r="C82" s="6">
+        <v>1.0250000000000001</v>
+      </c>
+      <c r="D82" s="6">
+        <v>1.03125</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="21">
+      <c r="A83">
+        <v>5166</v>
+      </c>
+      <c r="B83" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" s="6">
+        <v>1.0951388888888889</v>
+      </c>
+      <c r="D83" s="6">
+        <v>1.0993055555555555</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="21">
+      <c r="A84">
+        <v>5234</v>
+      </c>
+      <c r="B84" t="s">
+        <v>14</v>
+      </c>
+      <c r="C84" s="6">
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="D84" s="6">
+        <v>1.3375000000000001</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="21">
+      <c r="A85">
+        <v>5237</v>
+      </c>
+      <c r="B85" t="s">
+        <v>14</v>
+      </c>
+      <c r="C85" s="6">
+        <v>1.3388888888888888</v>
+      </c>
+      <c r="D85" s="6">
+        <v>1.3416666666666668</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="21">
+      <c r="A86">
+        <v>5301</v>
+      </c>
+      <c r="B86" t="s">
+        <v>14</v>
+      </c>
+      <c r="C86" s="6">
+        <v>1.5118055555555554</v>
+      </c>
+      <c r="D86" s="6">
+        <v>1.5159722222222223</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="42">
+      <c r="A87">
+        <v>5335</v>
+      </c>
+      <c r="B87" t="s">
+        <v>14</v>
+      </c>
+      <c r="C87" s="6">
+        <v>1.6027777777777779</v>
+      </c>
+      <c r="D87" s="6">
+        <v>1.6118055555555555</v>
+      </c>
+      <c r="E87" s="5" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="21">
+      <c r="A88">
+        <v>5472</v>
+      </c>
+      <c r="B88" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" s="7">
+        <v>8.4027777777777771E-2</v>
+      </c>
+      <c r="D88" s="7">
+        <v>9.0277777777777776E-2</v>
+      </c>
+      <c r="E88" s="5" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="21">
+      <c r="A89">
+        <v>5612</v>
+      </c>
+      <c r="B89" t="s">
+        <v>9</v>
+      </c>
+      <c r="C89" s="6">
+        <v>1.2541666666666667</v>
+      </c>
+      <c r="D89" s="6">
+        <v>1.2652777777777777</v>
+      </c>
+      <c r="E89" s="5" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="21">
+      <c r="A90">
+        <v>5753</v>
+      </c>
+      <c r="B90" t="s">
+        <v>31</v>
+      </c>
+      <c r="C90" s="7">
+        <v>0.15833333333333333</v>
+      </c>
+      <c r="D90" s="7">
+        <v>0.16111111111111112</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="21">
+      <c r="A91">
+        <v>5776</v>
+      </c>
+      <c r="B91" t="s">
+        <v>31</v>
+      </c>
+      <c r="C91" s="6">
+        <v>1.2347222222222223</v>
+      </c>
+      <c r="D91" s="6">
+        <v>1.2361111111111112</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="21">
+      <c r="A92">
+        <v>5793</v>
+      </c>
+      <c r="B92" t="s">
+        <v>16</v>
+      </c>
+      <c r="C92" s="7">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="D92" s="7">
+        <v>6.3888888888888884E-2</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="21">
+      <c r="A93">
+        <v>5852</v>
+      </c>
+      <c r="B93" t="s">
+        <v>16</v>
+      </c>
+      <c r="C93" s="7">
+        <v>0.21041666666666667</v>
+      </c>
+      <c r="D93" s="7">
+        <v>0.21597222222222223</v>
+      </c>
+      <c r="E93" s="5" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="21">
+      <c r="A94">
+        <v>6243</v>
+      </c>
+      <c r="B94" t="s">
+        <v>10</v>
+      </c>
+      <c r="C94" s="7">
+        <v>0.19375000000000001</v>
+      </c>
+      <c r="D94" s="7">
+        <v>0.19722222222222222</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="21">
+      <c r="A95">
+        <v>6331</v>
+      </c>
+      <c r="B95" t="s">
+        <v>10</v>
+      </c>
+      <c r="C95" s="7">
+        <v>0.40625</v>
+      </c>
+      <c r="D95" s="7">
+        <v>0.41250000000000003</v>
+      </c>
+      <c r="E95" s="5" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="21">
+      <c r="A96">
+        <v>6434</v>
+      </c>
+      <c r="B96" t="s">
+        <v>10</v>
+      </c>
+      <c r="C96" s="7">
+        <v>0.7583333333333333</v>
+      </c>
+      <c r="D96" s="7">
+        <v>0.76736111111111116</v>
+      </c>
+      <c r="E96" s="5" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="21">
+      <c r="A97">
+        <v>6510</v>
+      </c>
+      <c r="B97" t="s">
+        <v>10</v>
+      </c>
+      <c r="C97" s="6">
+        <v>1.0305555555555557</v>
+      </c>
+      <c r="D97" s="6">
+        <v>1.0347222222222221</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="21">
+      <c r="A98">
+        <v>6531</v>
+      </c>
+      <c r="B98" t="s">
+        <v>10</v>
+      </c>
+      <c r="C98" s="6">
+        <v>1.0777777777777777</v>
+      </c>
+      <c r="D98" s="6">
+        <v>1.0833333333333333</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="42">
+      <c r="A99">
+        <v>6709</v>
+      </c>
+      <c r="B99" t="s">
+        <v>10</v>
+      </c>
+      <c r="C99" s="6">
+        <v>1.5895833333333333</v>
+      </c>
+      <c r="D99" s="6">
+        <v>1.6006944444444444</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="21">
+      <c r="A100">
+        <v>6739</v>
+      </c>
+      <c r="B100" t="s">
+        <v>10</v>
+      </c>
+      <c r="C100" s="6">
+        <v>1.6506944444444445</v>
+      </c>
+      <c r="D100" s="6">
+        <v>1.653472222222222</v>
+      </c>
+      <c r="E100" s="5" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="21">
+      <c r="A101">
+        <v>6777</v>
+      </c>
+      <c r="B101" t="s">
+        <v>10</v>
+      </c>
+      <c r="C101" s="6">
+        <v>1.7145833333333333</v>
+      </c>
+      <c r="D101" s="6">
+        <v>1.7173611111111111</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>367</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H101">
+    <sortCondition ref="B2:B101"/>
+    <sortCondition ref="C2:C101"/>
+  </sortState>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60EE851F-A761-7B43-AAB8-B9484D09B5F1}">
   <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
@@ -3311,7 +5463,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="21">
+    <row r="6" spans="1:8" ht="42">
       <c r="A6">
         <v>511</v>
       </c>
@@ -3326,6 +5478,12 @@
       </c>
       <c r="E6" s="5" t="s">
         <v>170</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="21">
@@ -3344,6 +5502,9 @@
       <c r="E7" s="5" t="s">
         <v>155</v>
       </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="63">
       <c r="A8">
@@ -3361,6 +5522,15 @@
       <c r="E8" s="5" t="s">
         <v>235</v>
       </c>
+      <c r="F8" t="s">
+        <v>318</v>
+      </c>
+      <c r="G8">
+        <v>1.4</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="21">
       <c r="A9">
@@ -3378,6 +5548,9 @@
       <c r="E9" s="5" t="s">
         <v>313</v>
       </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="21">
       <c r="A10">
@@ -3395,6 +5568,9 @@
       <c r="E10" s="5" t="s">
         <v>61</v>
       </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="21">
       <c r="A11">
@@ -3412,6 +5588,9 @@
       <c r="E11" s="5" t="s">
         <v>27</v>
       </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="21">
       <c r="A12">
@@ -3429,6 +5608,9 @@
       <c r="E12" s="5" t="s">
         <v>115</v>
       </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="21">
       <c r="A13">
@@ -3446,6 +5628,9 @@
       <c r="E13" s="5" t="s">
         <v>191</v>
       </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="21">
       <c r="A14">
@@ -3463,6 +5648,9 @@
       <c r="E14" s="5" t="s">
         <v>103</v>
       </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="21">
       <c r="A15">
@@ -3480,6 +5668,9 @@
       <c r="E15" s="5" t="s">
         <v>176</v>
       </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="21">
       <c r="A16">
@@ -3497,8 +5688,11 @@
       <c r="E16" s="5" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="21">
+      <c r="F16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="21">
       <c r="A17">
         <v>1554</v>
       </c>
@@ -3514,8 +5708,11 @@
       <c r="E17" s="5" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="21">
+      <c r="F17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="21">
       <c r="A18">
         <v>1569</v>
       </c>
@@ -3531,8 +5728,11 @@
       <c r="E18" s="5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="21">
+      <c r="F18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="21">
       <c r="A19">
         <v>1615</v>
       </c>
@@ -3548,8 +5748,11 @@
       <c r="E19" s="5" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="21">
+      <c r="F19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="21">
       <c r="A20">
         <v>1694</v>
       </c>
@@ -3565,8 +5768,11 @@
       <c r="E20" s="5" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="21">
+      <c r="F20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="21">
       <c r="A21">
         <v>1703</v>
       </c>
@@ -3582,8 +5788,11 @@
       <c r="E21" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="21">
+      <c r="F21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="21">
       <c r="A22">
         <v>1730</v>
       </c>
@@ -3597,10 +5806,16 @@
         <v>271</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="21">
+        <v>320</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="21">
       <c r="A23">
         <v>1864</v>
       </c>
@@ -3616,8 +5831,11 @@
       <c r="E23" s="5" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="21">
+      <c r="F23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="21">
       <c r="A24">
         <v>1922</v>
       </c>
@@ -3631,10 +5849,13 @@
         <v>51</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="21">
+        <v>322</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="21">
       <c r="A25">
         <v>1934</v>
       </c>
@@ -3650,8 +5871,14 @@
       <c r="E25" s="5" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="21">
+      <c r="F25">
+        <v>2</v>
+      </c>
+      <c r="G25">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="21">
       <c r="A26">
         <v>2034</v>
       </c>
@@ -3667,8 +5894,11 @@
       <c r="E26" s="5" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="21">
+      <c r="F26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="21">
       <c r="A27">
         <v>2080</v>
       </c>
@@ -3684,8 +5914,11 @@
       <c r="E27" s="5" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="21">
+      <c r="F27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="21">
       <c r="A28">
         <v>2098</v>
       </c>
@@ -3701,8 +5934,11 @@
       <c r="E28" s="5" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="21">
+      <c r="F28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="21">
       <c r="A29">
         <v>2107</v>
       </c>
@@ -3718,8 +5954,11 @@
       <c r="E29" s="5" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="21">
+      <c r="F29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="21">
       <c r="A30">
         <v>2132</v>
       </c>
@@ -3735,8 +5974,11 @@
       <c r="E30" s="5" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="21">
+      <c r="F30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="21">
       <c r="A31">
         <v>2155</v>
       </c>
@@ -3752,8 +5994,11 @@
       <c r="E31" s="5" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" ht="21">
+      <c r="F31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="21">
       <c r="A32">
         <v>2323</v>
       </c>
@@ -3769,8 +6014,11 @@
       <c r="E32" s="5" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="42">
+      <c r="F32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="42">
       <c r="A33">
         <v>2576</v>
       </c>
@@ -3786,8 +6034,11 @@
       <c r="E33" s="5" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="42">
+      <c r="F33" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="42">
       <c r="A34">
         <v>2585</v>
       </c>
@@ -3803,8 +6054,11 @@
       <c r="E34" s="5" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="21">
+      <c r="F34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="21">
       <c r="A35">
         <v>2650</v>
       </c>
@@ -3820,8 +6074,11 @@
       <c r="E35" s="5" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="21">
+      <c r="F35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="21">
       <c r="A36">
         <v>2678</v>
       </c>
@@ -3837,8 +6094,11 @@
       <c r="E36" s="5" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="21">
+      <c r="F36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="21">
       <c r="A37">
         <v>2764</v>
       </c>
@@ -3854,8 +6114,11 @@
       <c r="E37" s="5" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="21">
+      <c r="F37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="21">
       <c r="A38">
         <v>2771</v>
       </c>
@@ -3871,8 +6134,11 @@
       <c r="E38" s="5" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="42">
+      <c r="F38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="42">
       <c r="A39">
         <v>2789</v>
       </c>
@@ -3888,8 +6154,11 @@
       <c r="E39" s="5" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" ht="21">
+      <c r="F39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="21">
       <c r="A40">
         <v>2865</v>
       </c>
@@ -3905,8 +6174,11 @@
       <c r="E40" s="5" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" ht="42">
+      <c r="F40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="42">
       <c r="A41">
         <v>2957</v>
       </c>
@@ -3922,8 +6194,11 @@
       <c r="E41" s="5" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" ht="21">
+      <c r="F41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="21">
       <c r="A42">
         <v>3114</v>
       </c>
@@ -3939,8 +6214,11 @@
       <c r="E42" s="5" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" ht="21">
+      <c r="F42">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="21">
       <c r="A43">
         <v>3121</v>
       </c>
@@ -3956,8 +6234,11 @@
       <c r="E43" s="5" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" ht="21">
+      <c r="F43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="21">
       <c r="A44">
         <v>3231</v>
       </c>
@@ -3973,8 +6254,11 @@
       <c r="E44" s="5" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" ht="21">
+      <c r="F44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="21">
       <c r="A45">
         <v>3257</v>
       </c>
@@ -3990,8 +6274,11 @@
       <c r="E45" s="5" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" ht="21">
+      <c r="F45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="21">
       <c r="A46">
         <v>3290</v>
       </c>
@@ -4007,8 +6294,11 @@
       <c r="E46" s="5" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="21">
+      <c r="F46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="21">
       <c r="A47">
         <v>3312</v>
       </c>
@@ -4024,8 +6314,11 @@
       <c r="E47" s="5" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" ht="21">
+      <c r="F47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="21">
       <c r="A48">
         <v>3381</v>
       </c>
@@ -4041,8 +6334,11 @@
       <c r="E48" s="5" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" ht="21">
+      <c r="F48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="21">
       <c r="A49">
         <v>3492</v>
       </c>
@@ -4058,8 +6354,11 @@
       <c r="E49" s="5" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" ht="21">
+      <c r="F49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="21">
       <c r="A50">
         <v>3509</v>
       </c>
@@ -4075,8 +6374,11 @@
       <c r="E50" s="5" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" ht="21">
+      <c r="F50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="21">
       <c r="A51">
         <v>3612</v>
       </c>
@@ -4092,8 +6394,11 @@
       <c r="E51" s="5" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" ht="21">
+      <c r="F51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="21">
       <c r="A52">
         <v>3662</v>
       </c>
@@ -4109,8 +6414,11 @@
       <c r="E52" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" ht="21">
+      <c r="F52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="21">
       <c r="A53">
         <v>3787</v>
       </c>
@@ -4126,8 +6434,11 @@
       <c r="E53" s="5" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" ht="21">
+      <c r="F53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="21">
       <c r="A54">
         <v>3837</v>
       </c>
@@ -4143,8 +6454,11 @@
       <c r="E54" s="5" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" ht="21">
+      <c r="F54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="21">
       <c r="A55">
         <v>3901</v>
       </c>
@@ -4160,8 +6474,11 @@
       <c r="E55" s="5" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" ht="21">
+      <c r="F55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="21">
       <c r="A56">
         <v>4094</v>
       </c>
@@ -4177,8 +6494,11 @@
       <c r="E56" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" ht="21">
+      <c r="F56">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="21">
       <c r="A57">
         <v>4119</v>
       </c>
@@ -4194,8 +6514,11 @@
       <c r="E57" s="5" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" ht="21">
+      <c r="F57">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="21">
       <c r="A58">
         <v>4204</v>
       </c>
@@ -4211,8 +6534,11 @@
       <c r="E58" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" ht="21">
+      <c r="F58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="21">
       <c r="A59">
         <v>4333</v>
       </c>
@@ -4228,8 +6554,11 @@
       <c r="E59" s="5" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" ht="21">
+      <c r="F59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="21">
       <c r="A60">
         <v>4498</v>
       </c>
@@ -4245,8 +6574,11 @@
       <c r="E60" s="5" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" ht="42">
+      <c r="F60">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="42">
       <c r="A61">
         <v>4541</v>
       </c>
@@ -4262,8 +6594,14 @@
       <c r="E61" s="5" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" ht="21">
+      <c r="F61" t="s">
+        <v>318</v>
+      </c>
+      <c r="H61" s="5" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="21">
       <c r="A62">
         <v>4556</v>
       </c>
@@ -4279,8 +6617,11 @@
       <c r="E62" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" ht="21">
+      <c r="F62" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="21">
       <c r="A63">
         <v>4608</v>
       </c>
@@ -4296,8 +6637,11 @@
       <c r="E63" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" ht="42">
+      <c r="F63">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="42">
       <c r="A64">
         <v>4649</v>
       </c>
@@ -4313,8 +6657,11 @@
       <c r="E64" s="5" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" ht="21">
+      <c r="F64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="21">
       <c r="A65">
         <v>4667</v>
       </c>
@@ -4330,8 +6677,11 @@
       <c r="E65" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" ht="21">
+      <c r="F65">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="21">
       <c r="A66">
         <v>4705</v>
       </c>
@@ -4347,8 +6697,11 @@
       <c r="E66" s="5" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" ht="21">
+      <c r="F66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="21">
       <c r="A67">
         <v>4866</v>
       </c>
@@ -4364,8 +6717,11 @@
       <c r="E67" s="5" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" ht="21">
+      <c r="F67">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="21">
       <c r="A68">
         <v>4898</v>
       </c>
@@ -4381,8 +6737,11 @@
       <c r="E68" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" ht="21">
+      <c r="F68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="21">
       <c r="A69">
         <v>5025</v>
       </c>
@@ -4398,8 +6757,11 @@
       <c r="E69" s="5" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" ht="21">
+      <c r="F69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="21">
       <c r="A70">
         <v>5033</v>
       </c>
@@ -4415,8 +6777,11 @@
       <c r="E70" s="5" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" ht="21">
+      <c r="F70">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="21">
       <c r="A71">
         <v>5058</v>
       </c>
@@ -4432,8 +6797,11 @@
       <c r="E71" s="5" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" ht="21">
+      <c r="F71">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" ht="21">
       <c r="A72">
         <v>5160</v>
       </c>
@@ -4449,8 +6817,11 @@
       <c r="E72" s="5" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" ht="21">
+      <c r="F72">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" ht="21">
       <c r="A73">
         <v>5170</v>
       </c>
@@ -4466,8 +6837,11 @@
       <c r="E73" s="5" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" ht="21">
+      <c r="F73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" ht="21">
       <c r="A74">
         <v>5204</v>
       </c>
@@ -4481,10 +6855,13 @@
         <v>96</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" ht="21">
+        <v>324</v>
+      </c>
+      <c r="F74">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="21">
       <c r="A75">
         <v>5275</v>
       </c>
@@ -4500,8 +6877,14 @@
       <c r="E75" s="5" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" ht="21">
+      <c r="F75" t="s">
+        <v>318</v>
+      </c>
+      <c r="H75" s="5" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" ht="21">
       <c r="A76">
         <v>5347</v>
       </c>
@@ -4517,8 +6900,11 @@
       <c r="E76" s="5" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" ht="21">
+      <c r="F76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="21">
       <c r="A77">
         <v>5371</v>
       </c>
@@ -4534,8 +6920,11 @@
       <c r="E77" s="5" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" ht="21">
+      <c r="F77">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="21">
       <c r="A78">
         <v>5538</v>
       </c>
@@ -4551,8 +6940,11 @@
       <c r="E78" s="5" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" ht="21">
+      <c r="F78">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" ht="21">
       <c r="A79">
         <v>5640</v>
       </c>
@@ -4568,8 +6960,11 @@
       <c r="E79" s="5" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" ht="21">
+      <c r="F79">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" ht="21">
       <c r="A80">
         <v>5663</v>
       </c>
@@ -4585,8 +6980,11 @@
       <c r="E80" s="5" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" ht="21">
+      <c r="F80" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" ht="21">
       <c r="A81">
         <v>5666</v>
       </c>
@@ -4606,7 +7004,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="21">
+    <row r="82" spans="1:8" ht="21">
       <c r="A82">
         <v>5712</v>
       </c>
@@ -4622,8 +7020,11 @@
       <c r="E82" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" ht="21">
+      <c r="F82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="21">
       <c r="A83">
         <v>5770</v>
       </c>
@@ -4640,7 +7041,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="21">
+    <row r="84" spans="1:8" ht="21">
       <c r="A84">
         <v>5924</v>
       </c>
@@ -4656,8 +7057,14 @@
       <c r="E84" s="5" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" ht="21">
+      <c r="F84">
+        <v>3</v>
+      </c>
+      <c r="H84" s="5" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" ht="21">
       <c r="A85">
         <v>5954</v>
       </c>
@@ -4673,8 +7080,11 @@
       <c r="E85" s="5" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" ht="21">
+      <c r="F85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" ht="21">
       <c r="A86">
         <v>5995</v>
       </c>
@@ -4690,8 +7100,11 @@
       <c r="E86" s="5" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" ht="21">
+      <c r="F86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" ht="21">
       <c r="A87">
         <v>6040</v>
       </c>
@@ -4707,8 +7120,14 @@
       <c r="E87" s="5" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" ht="21">
+      <c r="F87">
+        <v>3</v>
+      </c>
+      <c r="H87" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" ht="21">
       <c r="A88">
         <v>6062</v>
       </c>
@@ -4724,8 +7143,14 @@
       <c r="E88" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" ht="21">
+      <c r="F88">
+        <v>1</v>
+      </c>
+      <c r="H88" s="5" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" ht="21">
       <c r="A89">
         <v>6068</v>
       </c>
@@ -4741,8 +7166,11 @@
       <c r="E89" s="5" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" ht="21">
+      <c r="F89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" ht="21">
       <c r="A90">
         <v>6119</v>
       </c>
@@ -4758,8 +7186,11 @@
       <c r="E90" s="5" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" ht="21">
+      <c r="F90">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" ht="21">
       <c r="A91">
         <v>6139</v>
       </c>
@@ -4775,8 +7206,14 @@
       <c r="E91" s="5" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" ht="21">
+      <c r="F91">
+        <v>1</v>
+      </c>
+      <c r="H91" s="5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" ht="21">
       <c r="A92">
         <v>6151</v>
       </c>
@@ -4792,8 +7229,11 @@
       <c r="E92" s="5" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" ht="21">
+      <c r="F92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" ht="21">
       <c r="A93">
         <v>6158</v>
       </c>
@@ -4809,8 +7249,11 @@
       <c r="E93" s="5" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" ht="21">
+      <c r="F93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" ht="21">
       <c r="A94">
         <v>6288</v>
       </c>
@@ -4826,8 +7269,11 @@
       <c r="E94" s="5" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" ht="21">
+      <c r="F94">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" ht="21">
       <c r="A95">
         <v>6377</v>
       </c>
@@ -4843,8 +7289,11 @@
       <c r="E95" s="5" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" ht="21">
+      <c r="F95">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" ht="21">
       <c r="A96">
         <v>6404</v>
       </c>
@@ -4860,8 +7309,11 @@
       <c r="E96" s="5" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" ht="21">
+      <c r="F96">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="21">
       <c r="A97">
         <v>6446</v>
       </c>
@@ -4877,8 +7329,11 @@
       <c r="E97" s="5" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" ht="21">
+      <c r="F97">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="21">
       <c r="A98">
         <v>6559</v>
       </c>
@@ -4894,8 +7349,11 @@
       <c r="E98" s="5" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" ht="21">
+      <c r="F98">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="21">
       <c r="A99">
         <v>6721</v>
       </c>
@@ -4911,8 +7369,11 @@
       <c r="E99" s="5" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" ht="21">
+      <c r="F99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="21">
       <c r="A100">
         <v>6810</v>
       </c>
@@ -4928,8 +7389,11 @@
       <c r="E100" s="5" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" ht="21">
+      <c r="F100">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="21">
       <c r="A101">
         <v>6881</v>
       </c>
@@ -4944,10 +7408,14 @@
       </c>
       <c r="E101" s="5" t="s">
         <v>112</v>
+      </c>
+      <c r="F101">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[WIP] add annotation resource add annotated results
</commit_message>
<xml_diff>
--- a/annotation_tool/annotation_template.xlsx
+++ b/annotation_tool/annotation_template.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/heste/workspace/sn-caption/annotation_tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC121F6F-2392-7541-93C6-496A58E39BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29306902-DA2E-B844-8155-87A5A0CD77FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14660" yWindow="-28180" windowWidth="33940" windowHeight="14020" activeTab="1" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
+    <workbookView xWindow="55000" yWindow="-9180" windowWidth="25600" windowHeight="14160" activeTab="2" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
   </bookViews>
   <sheets>
-    <sheet name="テンプレート" sheetId="4" r:id="rId1"/>
+    <sheet name="テンプレート_seed42" sheetId="4" r:id="rId1"/>
     <sheet name="テンプレート_seed10" sheetId="6" r:id="rId2"/>
-    <sheet name="moriy" sheetId="5" r:id="rId3"/>
+    <sheet name="moriy_seed42" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_10_denoised_1_tokenized_224p_annotation" localSheetId="1">テンプレート_seed10!$A$1:$H$101</definedName>
-    <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="2">moriy!$A$1:$H$101</definedName>
-    <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="0">テンプレート!$A$1:$H$101</definedName>
+    <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="2">moriy_seed42!$A$1:$H$101</definedName>
+    <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="0">テンプレート_seed42!$A$1:$H$101</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="435">
   <si>
     <t>id</t>
   </si>
@@ -1112,16 +1112,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>付加的情報混じりの感想</t>
-    <rPh sb="0" eb="5">
-      <t xml:space="preserve">フカテキジョウホウ </t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t xml:space="preserve">マジリノカンソウ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>迷</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -1140,309 +1130,393 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>ちょいノイズ？</t>
+    <t>Now a idea.</t>
+  </si>
+  <si>
+    <t>He's smart because he's a fake.</t>
+  </si>
+  <si>
+    <t>It's Alaba and Alonso at the heart of that by in defence so it is very much unfamiliar looking defensive line for the home side.</t>
+  </si>
+  <si>
+    <t>When we say holding in the box, we're not talking about a foul now.</t>
+  </si>
+  <si>
+    <t>2015-02-15 - 14-30 AC Milan 1 - 1 Empoli</t>
+  </si>
+  <si>
+    <t>...Menes really is the... ...inspiration for Milan... ...at the moment.</t>
+  </si>
+  <si>
+    <t>Dani Alves is trying to score.</t>
+  </si>
+  <si>
+    <t>Alexander has a problem with the ball.</t>
+  </si>
+  <si>
+    <t>He became much coveted after his time at Southampton, which began here.</t>
+  </si>
+  <si>
+    <t>Mkhmedi.</t>
+  </si>
+  <si>
+    <t>The number 19 Ivan Cavallero.</t>
+  </si>
+  <si>
+    <t>Ronaldo got a hat-trick that day as I mentioned.</t>
+  </si>
+  <si>
+    <t>Marcelo wanted to leave first for Kroos, he gives it directly to the rival.</t>
+  </si>
+  <si>
+    <t>Now the counter-attack.</t>
+  </si>
+  <si>
+    <t>He's been controlling all these things.</t>
+  </si>
+  <si>
+    <t>Kjezo again.</t>
+  </si>
+  <si>
+    <t>Paderborn from the beginning with a clear defense concept.</t>
+  </si>
+  <si>
+    <t>Koke.</t>
+  </si>
+  <si>
+    <t>He shot from a distance.</t>
+  </si>
+  <si>
+    <t>The problem for FC Barcelona is Alventosa's presence.</t>
+  </si>
+  <si>
+    <t>Calcio is returning, which, I think, all fans of the series are very happy about.</t>
+  </si>
+  <si>
+    <t>Hey!</t>
+  </si>
+  <si>
+    <t>Hasn't yet been a break in play.</t>
+  </si>
+  <si>
+    <t>Dani Alves is playing with a traditional Juventus' style.</t>
+  </si>
+  <si>
+    <t>I don't think so.</t>
+  </si>
+  <si>
+    <t>The Zinedine Zidane team are trying to get the ball out, Toni Kroos is looking for it, it's a bad pass.</t>
+  </si>
+  <si>
+    <t>Now Hulk up.</t>
+  </si>
+  <si>
+    <t>And then the non-rule climbing handball.</t>
+  </si>
+  <si>
+    <t>Vidal.</t>
+  </si>
+  <si>
+    <t>Does the little pass inside.</t>
+  </si>
+  <si>
+    <t>Depor will come out obviously looking to defend their goal especially over the first 20 minutes or so.</t>
+  </si>
+  <si>
+    <t>There was no flag.</t>
+  </si>
+  <si>
+    <t>Chelsea in those wide areas.</t>
+  </si>
+  <si>
+    <t>Everything you can win by 1-0 is always very dangerous.</t>
+  </si>
+  <si>
+    <t>The player of the German national team scores the first Juventus ball in the new season.</t>
+  </si>
+  <si>
+    <t>So good start here for the Galicians.</t>
+  </si>
+  <si>
+    <t>Rakitic.</t>
+  </si>
+  <si>
+    <t>Another long ball.</t>
+  </si>
+  <si>
+    <t>Mario Götze is left to Stefan Ilsenker.</t>
+  </si>
+  <si>
+    <t>Nacho outside to the Brazilian left back.</t>
+  </si>
+  <si>
+    <t>Good wall from Bernardeschi.</t>
+  </si>
+  <si>
+    <t>Shaquille has failed.</t>
+  </si>
+  <si>
+    <t>Burak is turning.</t>
+  </si>
+  <si>
+    <t>He scored a yellow-red goal in Lviv.</t>
+  </si>
+  <si>
+    <t>Ribéry, quickly with Lewandowski.</t>
+  </si>
+  <si>
+    <t>He shoots the header.</t>
+  </si>
+  <si>
+    <t>I think he's capable of it.</t>
+  </si>
+  <si>
+    <t>That's why the great good of European football covered his signature.</t>
+  </si>
+  <si>
+    <t>Trapp!</t>
+  </si>
+  <si>
+    <t>But I think everybody knew Cristiano Ronaldo was going to go for goal from that position.</t>
+  </si>
+  <si>
+    <t>It's going to move.</t>
+  </si>
+  <si>
+    <t>And got themselves right back in the game.</t>
+  </si>
+  <si>
+    <t>Although it's just going to beat Marquinhos.</t>
+  </si>
+  <si>
+    <t>Chalhanoglu helps it on towards Kiesling.</t>
+  </si>
+  <si>
+    <t>I must say that they are taking advantage of the change of rules.</t>
+  </si>
+  <si>
+    <t>This is not good for PSG.</t>
+  </si>
+  <si>
+    <t>The ball continues to be on the left side.</t>
+  </si>
+  <si>
+    <t>Hilbert under pressure from Costa.</t>
+  </si>
+  <si>
+    <t>Ventus again.</t>
+  </si>
+  <si>
+    <t>Intuitive Marcelo, that opening by Fran Beltran, made Kevin doubt just enough so that no one touched the ball.</t>
+  </si>
+  <si>
+    <t>Meha is actually the right one on the ball.</t>
+  </si>
+  <si>
+    <t>In a practically full Camp Nou.</t>
+  </si>
+  <si>
+    <t>They say he was on the list of Aurelio de Laurentiis, the president of Naples, after the sale of Gonçalo Higuain.</t>
+  </si>
+  <si>
+    <t>Penalty shout at both ends.</t>
+  </si>
+  <si>
+    <t>It's a very tight ball.</t>
+  </si>
+  <si>
+    <t>You have to say Arsenal have done well with that.</t>
+  </si>
+  <si>
+    <t>Lobotka.</t>
+  </si>
+  <si>
+    <t>First from Kacunga and last from Lukas Rupp.</t>
+  </si>
+  <si>
+    <t>Laura now in possession looking for a free kick that doesn't come.</t>
+  </si>
+  <si>
+    <t>Lowry lost track of it.</t>
+  </si>
+  <si>
+    <t>Vermaelen for Macerano.</t>
+  </si>
+  <si>
+    <t>They were incredible.</t>
+  </si>
+  <si>
+    <t>Teams that will consider those positions to be the minimum of their domestic requirements for this season again.</t>
+  </si>
+  <si>
+    <t>It was not his natural position, but he had many casualties in that demarcation.</t>
+  </si>
+  <si>
+    <t>And now the card is being shown.</t>
+  </si>
+  <si>
+    <t>Isco, little flick to the back post.</t>
+  </si>
+  <si>
+    <t>Because there are many people who want to buy an Italian star.</t>
+  </si>
+  <si>
+    <t>I think I have the statistics, and Ivanovic has scored 27 goals since August 2010.</t>
+  </si>
+  <si>
+    <t>I think he trusts a lot that he will have space and that he can kill him on the counter.</t>
+  </si>
+  <si>
+    <t>I think he's a good player, Adam Lallana.</t>
+  </si>
+  <si>
+    <t>And he gives them stability in the heart of the midfield.</t>
+  </si>
+  <si>
+    <t>Burak.</t>
+  </si>
+  <si>
+    <t>Maybe they changed their mind.</t>
+  </si>
+  <si>
+    <t>You can whistle a foul, you can not whistle a foul and therefore the VAR does not enter there.</t>
+  </si>
+  <si>
+    <t>Cristiano Ronaldo's goal is repeated.</t>
+  </si>
+  <si>
+    <t>Sergi Roberto getting ready for a shot.</t>
+  </si>
+  <si>
+    <t>Aspire Cueta.</t>
+  </si>
+  <si>
+    <t>Keline.</t>
+  </si>
+  <si>
+    <t>This is what we are saying.</t>
+  </si>
+  <si>
+    <t>This is a very powerful football game that the team of André Breitenreiter offers in this early phase, but they are set for it.</t>
+  </si>
+  <si>
+    <t>Atletico Madrid scored the twelfth goal.</t>
+  </si>
+  <si>
+    <t>And he didn't just know, he scored a perfect goal.</t>
+  </si>
+  <si>
+    <t>On Cruz brings him down it'll be another free kick they'll have to be taken a few meters back.</t>
+  </si>
+  <si>
+    <t>It's a failed interception, Ronaldo has Benzema inside, can't get around Lopo.</t>
+  </si>
+  <si>
+    <t>All attacks are thrown in by the Spanish ex-world champion.</t>
+  </si>
+  <si>
+    <t>The pitch is strangely in poor condition normally early on in the season.</t>
+  </si>
+  <si>
+    <t>He saves the ball.</t>
+  </si>
+  <si>
+    <t>Cristiano Ronaldo.</t>
+  </si>
+  <si>
+    <t>迷。付加的情報混じりの感想</t>
+    <rPh sb="0" eb="1">
+      <t xml:space="preserve">マヨッタ </t>
+    </rPh>
+    <rPh sb="2" eb="7">
+      <t xml:space="preserve">フカテキジョウホウ </t>
+    </rPh>
+    <rPh sb="7" eb="8">
+      <t xml:space="preserve">マジリノカンソウ </t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>Now a idea.</t>
-  </si>
-  <si>
-    <t>He's smart because he's a fake.</t>
-  </si>
-  <si>
-    <t>It's Alaba and Alonso at the heart of that by in defence so it is very much unfamiliar looking defensive line for the home side.</t>
-  </si>
-  <si>
-    <t>When we say holding in the box, we're not talking about a foul now.</t>
-  </si>
-  <si>
-    <t>2015-02-15 - 14-30 AC Milan 1 - 1 Empoli</t>
-  </si>
-  <si>
-    <t>...Menes really is the... ...inspiration for Milan... ...at the moment.</t>
-  </si>
-  <si>
-    <t>Dani Alves is trying to score.</t>
-  </si>
-  <si>
-    <t>Alexander has a problem with the ball.</t>
-  </si>
-  <si>
-    <t>He became much coveted after his time at Southampton, which began here.</t>
-  </si>
-  <si>
-    <t>Mkhmedi.</t>
-  </si>
-  <si>
-    <t>The number 19 Ivan Cavallero.</t>
-  </si>
-  <si>
-    <t>Ronaldo got a hat-trick that day as I mentioned.</t>
-  </si>
-  <si>
-    <t>Marcelo wanted to leave first for Kroos, he gives it directly to the rival.</t>
-  </si>
-  <si>
-    <t>Now the counter-attack.</t>
-  </si>
-  <si>
-    <t>He's been controlling all these things.</t>
-  </si>
-  <si>
-    <t>Kjezo again.</t>
-  </si>
-  <si>
-    <t>Paderborn from the beginning with a clear defense concept.</t>
-  </si>
-  <si>
-    <t>Koke.</t>
-  </si>
-  <si>
-    <t>He shot from a distance.</t>
-  </si>
-  <si>
-    <t>The problem for FC Barcelona is Alventosa's presence.</t>
-  </si>
-  <si>
-    <t>Calcio is returning, which, I think, all fans of the series are very happy about.</t>
-  </si>
-  <si>
-    <t>Hey!</t>
-  </si>
-  <si>
-    <t>Hasn't yet been a break in play.</t>
-  </si>
-  <si>
-    <t>Dani Alves is playing with a traditional Juventus' style.</t>
-  </si>
-  <si>
-    <t>I don't think so.</t>
-  </si>
-  <si>
-    <t>The Zinedine Zidane team are trying to get the ball out, Toni Kroos is looking for it, it's a bad pass.</t>
-  </si>
-  <si>
-    <t>Now Hulk up.</t>
-  </si>
-  <si>
-    <t>And then the non-rule climbing handball.</t>
-  </si>
-  <si>
-    <t>Vidal.</t>
-  </si>
-  <si>
-    <t>Does the little pass inside.</t>
-  </si>
-  <si>
-    <t>Depor will come out obviously looking to defend their goal especially over the first 20 minutes or so.</t>
-  </si>
-  <si>
-    <t>There was no flag.</t>
-  </si>
-  <si>
-    <t>Chelsea in those wide areas.</t>
-  </si>
-  <si>
-    <t>Everything you can win by 1-0 is always very dangerous.</t>
-  </si>
-  <si>
-    <t>The player of the German national team scores the first Juventus ball in the new season.</t>
-  </si>
-  <si>
-    <t>So good start here for the Galicians.</t>
-  </si>
-  <si>
-    <t>Rakitic.</t>
-  </si>
-  <si>
-    <t>Another long ball.</t>
-  </si>
-  <si>
-    <t>Mario Götze is left to Stefan Ilsenker.</t>
-  </si>
-  <si>
-    <t>Nacho outside to the Brazilian left back.</t>
-  </si>
-  <si>
-    <t>Good wall from Bernardeschi.</t>
-  </si>
-  <si>
-    <t>Shaquille has failed.</t>
-  </si>
-  <si>
-    <t>Burak is turning.</t>
-  </si>
-  <si>
-    <t>He scored a yellow-red goal in Lviv.</t>
-  </si>
-  <si>
-    <t>Ribéry, quickly with Lewandowski.</t>
-  </si>
-  <si>
-    <t>He shoots the header.</t>
-  </si>
-  <si>
-    <t>I think he's capable of it.</t>
-  </si>
-  <si>
-    <t>That's why the great good of European football covered his signature.</t>
-  </si>
-  <si>
-    <t>Trapp!</t>
-  </si>
-  <si>
-    <t>But I think everybody knew Cristiano Ronaldo was going to go for goal from that position.</t>
-  </si>
-  <si>
-    <t>It's going to move.</t>
-  </si>
-  <si>
-    <t>And got themselves right back in the game.</t>
-  </si>
-  <si>
-    <t>Although it's just going to beat Marquinhos.</t>
-  </si>
-  <si>
-    <t>Chalhanoglu helps it on towards Kiesling.</t>
-  </si>
-  <si>
-    <t>I must say that they are taking advantage of the change of rules.</t>
-  </si>
-  <si>
-    <t>This is not good for PSG.</t>
-  </si>
-  <si>
-    <t>The ball continues to be on the left side.</t>
-  </si>
-  <si>
-    <t>Hilbert under pressure from Costa.</t>
-  </si>
-  <si>
-    <t>Ventus again.</t>
-  </si>
-  <si>
-    <t>Intuitive Marcelo, that opening by Fran Beltran, made Kevin doubt just enough so that no one touched the ball.</t>
-  </si>
-  <si>
-    <t>Meha is actually the right one on the ball.</t>
-  </si>
-  <si>
-    <t>In a practically full Camp Nou.</t>
-  </si>
-  <si>
-    <t>They say he was on the list of Aurelio de Laurentiis, the president of Naples, after the sale of Gonçalo Higuain.</t>
-  </si>
-  <si>
-    <t>Penalty shout at both ends.</t>
-  </si>
-  <si>
-    <t>It's a very tight ball.</t>
-  </si>
-  <si>
-    <t>You have to say Arsenal have done well with that.</t>
-  </si>
-  <si>
-    <t>Lobotka.</t>
-  </si>
-  <si>
-    <t>First from Kacunga and last from Lukas Rupp.</t>
-  </si>
-  <si>
-    <t>Laura now in possession looking for a free kick that doesn't come.</t>
-  </si>
-  <si>
-    <t>Lowry lost track of it.</t>
-  </si>
-  <si>
-    <t>Vermaelen for Macerano.</t>
-  </si>
-  <si>
-    <t>They were incredible.</t>
-  </si>
-  <si>
-    <t>Teams that will consider those positions to be the minimum of their domestic requirements for this season again.</t>
-  </si>
-  <si>
-    <t>It was not his natural position, but he had many casualties in that demarcation.</t>
-  </si>
-  <si>
-    <t>And now the card is being shown.</t>
-  </si>
-  <si>
-    <t>Isco, little flick to the back post.</t>
-  </si>
-  <si>
-    <t>Because there are many people who want to buy an Italian star.</t>
-  </si>
-  <si>
-    <t>I think I have the statistics, and Ivanovic has scored 27 goals since August 2010.</t>
-  </si>
-  <si>
-    <t>I think he trusts a lot that he will have space and that he can kill him on the counter.</t>
-  </si>
-  <si>
-    <t>I think he's a good player, Adam Lallana.</t>
-  </si>
-  <si>
-    <t>And he gives them stability in the heart of the midfield.</t>
-  </si>
-  <si>
-    <t>Burak.</t>
-  </si>
-  <si>
-    <t>Maybe they changed their mind.</t>
-  </si>
-  <si>
-    <t>You can whistle a foul, you can not whistle a foul and therefore the VAR does not enter there.</t>
-  </si>
-  <si>
-    <t>Cristiano Ronaldo's goal is repeated.</t>
-  </si>
-  <si>
-    <t>Sergi Roberto getting ready for a shot.</t>
-  </si>
-  <si>
-    <t>Aspire Cueta.</t>
-  </si>
-  <si>
-    <t>Keline.</t>
-  </si>
-  <si>
-    <t>This is what we are saying.</t>
-  </si>
-  <si>
-    <t>This is a very powerful football game that the team of André Breitenreiter offers in this early phase, but they are set for it.</t>
-  </si>
-  <si>
-    <t>Atletico Madrid scored the twelfth goal.</t>
-  </si>
-  <si>
-    <t>And he didn't just know, he scored a perfect goal.</t>
-  </si>
-  <si>
-    <t>On Cruz brings him down it'll be another free kick they'll have to be taken a few meters back.</t>
-  </si>
-  <si>
-    <t>It's a failed interception, Ronaldo has Benzema inside, can't get around Lopo.</t>
-  </si>
-  <si>
-    <t>All attacks are thrown in by the Spanish ex-world champion.</t>
-  </si>
-  <si>
-    <t>The pitch is strangely in poor condition normally early on in the season.</t>
-  </si>
-  <si>
-    <t>He saves the ball.</t>
-  </si>
-  <si>
-    <t>Cristiano Ronaldo.</t>
+    <r>
+      <t xml:space="preserve">We are watching again Atletico Madrid </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>In 2010</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In UEFA European League　（最近洗練されていたアトレティコだが、この試合は昔のようなよくない調子、という意味で捉えた）</t>
+    </r>
+    <rPh sb="71" eb="75">
+      <t xml:space="preserve">サイキンセンレン </t>
+    </rPh>
+    <rPh sb="94" eb="95">
+      <t xml:space="preserve">ムカシノヨウナ </t>
+    </rPh>
+    <rPh sb="103" eb="105">
+      <t xml:space="preserve">チョウシ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1 3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ファールシーンで、削られた側がうまくいなしている状況</t>
+    <rPh sb="9" eb="10">
+      <t xml:space="preserve">ケズラレタガワ </t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t xml:space="preserve">ジョウキョウ </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>完全な文章ではない</t>
+    <rPh sb="0" eb="2">
+      <t xml:space="preserve">カンゼン </t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>What an impression he's made on Bayern and what a remarkable achievement it would be if he could produce that unprecedented fourth consecutive Bundesliga title.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2016-08-14 - 18-00 Arsenal 3 - 4 Liverpool</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Sneijder.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2015-08-29 - 19-30 Bayern Munich 3 - 0 Bayer Leverkusen</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1455,6 +1529,15 @@
       <sz val="6"/>
       <name val="游ゴシック"/>
       <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
@@ -3642,7 +3725,7 @@
         <v>0.17222222222222225</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="21">
@@ -3659,7 +3742,7 @@
         <v>0.25</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="21">
@@ -3676,7 +3759,7 @@
         <v>2.7083333333333334E-2</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="21">
@@ -3693,7 +3776,7 @@
         <v>8.7500000000000008E-2</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="21">
@@ -3710,7 +3793,7 @@
         <v>0.21319444444444444</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="21">
@@ -3727,7 +3810,7 @@
         <v>0.29097222222222224</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="21">
@@ -3744,7 +3827,7 @@
         <v>0.31666666666666665</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="21">
@@ -3761,7 +3844,7 @@
         <v>0.35486111111111113</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="21">
@@ -3778,7 +3861,7 @@
         <v>0.51111111111111118</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="21">
@@ -3795,7 +3878,7 @@
         <v>0.53055555555555556</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="21">
@@ -3812,7 +3895,7 @@
         <v>0.64930555555555558</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="21">
@@ -3829,7 +3912,7 @@
         <v>0.86875000000000002</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="21">
@@ -3846,7 +3929,7 @@
         <v>0.9277777777777777</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="21">
@@ -3863,7 +3946,7 @@
         <v>0.9868055555555556</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="21">
@@ -3880,7 +3963,7 @@
         <v>1.0395833333333333</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="21">
@@ -3897,7 +3980,7 @@
         <v>1.1937499999999999</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="21">
@@ -3905,7 +3988,7 @@
         <v>760</v>
       </c>
       <c r="B18" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C18" s="7">
         <v>0.72777777777777775</v>
@@ -3914,7 +3997,7 @@
         <v>0.73888888888888893</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="21">
@@ -3931,7 +4014,7 @@
         <v>5.2777777777777778E-2</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="42">
@@ -3948,7 +4031,7 @@
         <v>0.77013888888888893</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="21">
@@ -3965,7 +4048,7 @@
         <v>0.79236111111111107</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="21">
@@ -3982,7 +4065,7 @@
         <v>1.6569444444444443</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="21">
@@ -3999,7 +4082,7 @@
         <v>1.6659722222222222</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="21">
@@ -4016,7 +4099,7 @@
         <v>1.6763888888888889</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="21">
@@ -4033,7 +4116,7 @@
         <v>1.6777777777777778</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="21">
@@ -4050,7 +4133,7 @@
         <v>1.8472222222222223</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="21">
@@ -4067,7 +4150,7 @@
         <v>8.1250000000000003E-2</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="21">
@@ -4084,7 +4167,7 @@
         <v>0.22083333333333333</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="21">
@@ -4101,7 +4184,7 @@
         <v>0.59166666666666667</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="21">
@@ -4118,7 +4201,7 @@
         <v>1.0111111111111111</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="21">
@@ -4135,7 +4218,7 @@
         <v>1.6458333333333333</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="21">
@@ -4152,7 +4235,7 @@
         <v>1.8263888888888891</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="21">
@@ -4169,7 +4252,7 @@
         <v>1.8729166666666668</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="21">
@@ -4186,7 +4269,7 @@
         <v>0.11875000000000001</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="21">
@@ -4203,7 +4286,7 @@
         <v>0.32708333333333334</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="21">
@@ -4220,7 +4303,7 @@
         <v>0.34375</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="21">
@@ -4237,7 +4320,7 @@
         <v>0.38680555555555557</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="21">
@@ -4254,7 +4337,7 @@
         <v>1.3472222222222223</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="21">
@@ -4271,7 +4354,7 @@
         <v>0.14583333333333334</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="21">
@@ -4288,7 +4371,7 @@
         <v>0.15694444444444444</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="21">
@@ -4305,7 +4388,7 @@
         <v>1.4118055555555555</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="21">
@@ -4322,7 +4405,7 @@
         <v>1.4958333333333333</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="21">
@@ -4339,7 +4422,7 @@
         <v>1.5895833333333333</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="42">
@@ -4356,7 +4439,7 @@
         <v>0.21319444444444444</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="21">
@@ -4373,7 +4456,7 @@
         <v>0.2722222222222222</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="21">
@@ -4390,7 +4473,7 @@
         <v>0.6069444444444444</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="21">
@@ -4407,7 +4490,7 @@
         <v>0.62777777777777777</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="21">
@@ -4424,7 +4507,7 @@
         <v>0.86944444444444446</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="21">
@@ -4441,7 +4524,7 @@
         <v>0.91249999999999998</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="21">
@@ -4458,7 +4541,7 @@
         <v>1.4861111111111109</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="21">
@@ -4475,7 +4558,7 @@
         <v>1.6465277777777778</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="42">
@@ -4492,7 +4575,7 @@
         <v>1.7138888888888888</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="21">
@@ -4509,7 +4592,7 @@
         <v>5.8333333333333327E-2</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="21">
@@ -4543,7 +4626,7 @@
         <v>0.47500000000000003</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="21">
@@ -4560,7 +4643,7 @@
         <v>0.53333333333333333</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="21">
@@ -4577,7 +4660,7 @@
         <v>1.3673611111111112</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="21">
@@ -4594,7 +4677,7 @@
         <v>1.6354166666666667</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="21">
@@ -4611,7 +4694,7 @@
         <v>1.7145833333333333</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="21">
@@ -4628,7 +4711,7 @@
         <v>1.7277777777777779</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="21">
@@ -4645,7 +4728,7 @@
         <v>1.7618055555555554</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="21">
@@ -4679,7 +4762,7 @@
         <v>0.3520833333333333</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="21">
@@ -4696,7 +4779,7 @@
         <v>0.50138888888888888</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="21">
@@ -4713,7 +4796,7 @@
         <v>0.92708333333333337</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="21">
@@ -4730,7 +4813,7 @@
         <v>0.99375000000000002</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="21">
@@ -4747,7 +4830,7 @@
         <v>1.0430555555555556</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="21">
@@ -4764,7 +4847,7 @@
         <v>1.1736111111111112</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="21">
@@ -4781,7 +4864,7 @@
         <v>7.9166666666666663E-2</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="21">
@@ -4798,7 +4881,7 @@
         <v>0.56319444444444444</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="21">
@@ -4815,7 +4898,7 @@
         <v>0.65555555555555556</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="21">
@@ -4832,7 +4915,7 @@
         <v>0.66875000000000007</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="21">
@@ -4849,7 +4932,7 @@
         <v>1.0777777777777777</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="21">
@@ -4866,7 +4949,7 @@
         <v>1.8694444444444445</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="21">
@@ -4883,7 +4966,7 @@
         <v>5.8333333333333327E-2</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="21">
@@ -4900,7 +4983,7 @@
         <v>7.7083333333333337E-2</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="21">
@@ -4917,7 +5000,7 @@
         <v>0.20486111111111113</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="21">
@@ -4934,7 +5017,7 @@
         <v>0.51388888888888895</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="21">
@@ -4968,7 +5051,7 @@
         <v>0.72222222222222221</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="21">
@@ -4985,7 +5068,7 @@
         <v>0.96250000000000002</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="21">
@@ -5002,7 +5085,7 @@
         <v>1.03125</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="21">
@@ -5019,7 +5102,7 @@
         <v>1.0993055555555555</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="21">
@@ -5036,7 +5119,7 @@
         <v>1.3375000000000001</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="21">
@@ -5053,7 +5136,7 @@
         <v>1.3416666666666668</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="21">
@@ -5070,7 +5153,7 @@
         <v>1.5159722222222223</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="42">
@@ -5087,7 +5170,7 @@
         <v>1.6118055555555555</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="21">
@@ -5104,7 +5187,7 @@
         <v>9.0277777777777776E-2</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="21">
@@ -5121,7 +5204,7 @@
         <v>1.2652777777777777</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="21">
@@ -5138,7 +5221,7 @@
         <v>0.16111111111111112</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="21">
@@ -5155,7 +5238,7 @@
         <v>1.2361111111111112</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="21">
@@ -5172,7 +5255,7 @@
         <v>6.3888888888888884E-2</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="21">
@@ -5189,7 +5272,7 @@
         <v>0.21597222222222223</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="94" spans="1:5" ht="21">
@@ -5206,7 +5289,7 @@
         <v>0.19722222222222222</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="21">
@@ -5223,7 +5306,7 @@
         <v>0.41250000000000003</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="21">
@@ -5240,7 +5323,7 @@
         <v>0.76736111111111116</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="21">
@@ -5257,7 +5340,7 @@
         <v>1.0347222222222221</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="21">
@@ -5274,7 +5357,7 @@
         <v>1.0833333333333333</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="42">
@@ -5291,7 +5374,7 @@
         <v>1.6006944444444444</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="21">
@@ -5308,7 +5391,7 @@
         <v>1.653472222222222</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="21">
@@ -5325,7 +5408,7 @@
         <v>1.7173611111111111</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -5347,8 +5430,9 @@
     <col min="2" max="2" width="53.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="80.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.85546875" style="5" customWidth="1"/>
+    <col min="6" max="6" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.85546875" customWidth="1"/>
+    <col min="8" max="8" width="44.140625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="21">
@@ -5875,7 +5959,7 @@
         <v>2</v>
       </c>
       <c r="G25">
-        <v>1.4</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="21">
@@ -6018,7 +6102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="42">
+    <row r="33" spans="1:7" ht="42">
       <c r="A33">
         <v>2576</v>
       </c>
@@ -6032,13 +6116,16 @@
         <v>300</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>301</v>
+        <v>431</v>
       </c>
       <c r="F33" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="42">
+      <c r="G33">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="42">
       <c r="A34">
         <v>2585</v>
       </c>
@@ -6057,8 +6144,11 @@
       <c r="F34">
         <v>2</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="21">
+      <c r="G34">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="21">
       <c r="A35">
         <v>2650</v>
       </c>
@@ -6078,7 +6168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="21">
+    <row r="36" spans="1:7" ht="21">
       <c r="A36">
         <v>2678</v>
       </c>
@@ -6098,7 +6188,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="21">
+    <row r="37" spans="1:7" ht="21">
       <c r="A37">
         <v>2764</v>
       </c>
@@ -6117,8 +6207,11 @@
       <c r="F37">
         <v>2</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="21">
+      <c r="G37">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="21">
       <c r="A38">
         <v>2771</v>
       </c>
@@ -6138,7 +6231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="42">
+    <row r="39" spans="1:7" ht="42">
       <c r="A39">
         <v>2789</v>
       </c>
@@ -6157,13 +6250,16 @@
       <c r="F39">
         <v>2</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="21">
+      <c r="G39">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="21">
       <c r="A40">
         <v>2865</v>
       </c>
       <c r="B40" t="s">
-        <v>12</v>
+        <v>434</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>148</v>
@@ -6177,8 +6273,11 @@
       <c r="F40">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="42">
+      <c r="G40">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="42">
       <c r="A41">
         <v>2957</v>
       </c>
@@ -6198,7 +6297,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="21">
+    <row r="42" spans="1:7" ht="21">
       <c r="A42">
         <v>3114</v>
       </c>
@@ -6218,7 +6317,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="21">
+    <row r="43" spans="1:7" ht="21">
       <c r="A43">
         <v>3121</v>
       </c>
@@ -6238,7 +6337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="21">
+    <row r="44" spans="1:7" ht="21">
       <c r="A44">
         <v>3231</v>
       </c>
@@ -6258,7 +6357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="21">
+    <row r="45" spans="1:7" ht="21">
       <c r="A45">
         <v>3257</v>
       </c>
@@ -6278,7 +6377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="21">
+    <row r="46" spans="1:7" ht="21">
       <c r="A46">
         <v>3290</v>
       </c>
@@ -6298,7 +6397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="21">
+    <row r="47" spans="1:7" ht="21">
       <c r="A47">
         <v>3312</v>
       </c>
@@ -6318,7 +6417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="21">
+    <row r="48" spans="1:7" ht="21">
       <c r="A48">
         <v>3381</v>
       </c>
@@ -6437,6 +6536,9 @@
       <c r="F53">
         <v>2</v>
       </c>
+      <c r="G53">
+        <v>2.2999999999999998</v>
+      </c>
     </row>
     <row r="54" spans="1:8" ht="21">
       <c r="A54">
@@ -6498,7 +6600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="21">
+    <row r="57" spans="1:8" ht="84">
       <c r="A57">
         <v>4119</v>
       </c>
@@ -6515,7 +6617,10 @@
         <v>226</v>
       </c>
       <c r="F57">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="H57" s="5" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="21">
@@ -6532,7 +6637,7 @@
         <v>66</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>67</v>
+        <v>433</v>
       </c>
       <c r="F58">
         <v>1</v>
@@ -6597,6 +6702,9 @@
       <c r="F61" t="s">
         <v>318</v>
       </c>
+      <c r="G61">
+        <v>3.3</v>
+      </c>
       <c r="H61" s="5" t="s">
         <v>323</v>
       </c>
@@ -6606,7 +6714,7 @@
         <v>4556</v>
       </c>
       <c r="B62" t="s">
-        <v>18</v>
+        <v>432</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>118</v>
@@ -6619,6 +6727,9 @@
       </c>
       <c r="F62" t="s">
         <v>318</v>
+      </c>
+      <c r="G62">
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="21">
@@ -6640,6 +6751,9 @@
       <c r="F63">
         <v>2</v>
       </c>
+      <c r="G63">
+        <v>1.1000000000000001</v>
+      </c>
     </row>
     <row r="64" spans="1:8" ht="42">
       <c r="A64">
@@ -6780,6 +6894,9 @@
       <c r="F70">
         <v>2</v>
       </c>
+      <c r="G70">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="71" spans="1:8" ht="21">
       <c r="A71">
@@ -6877,11 +6994,11 @@
       <c r="E75" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="F75" t="s">
-        <v>318</v>
+      <c r="F75">
+        <v>3</v>
       </c>
       <c r="H75" s="5" t="s">
-        <v>325</v>
+        <v>426</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="21">
@@ -6923,6 +7040,9 @@
       <c r="F77">
         <v>2</v>
       </c>
+      <c r="G77">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="78" spans="1:8" ht="21">
       <c r="A78">
@@ -6964,7 +7084,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="21">
+    <row r="80" spans="1:8" ht="42">
       <c r="A80">
         <v>5663</v>
       </c>
@@ -6981,7 +7101,10 @@
         <v>197</v>
       </c>
       <c r="F80" t="s">
-        <v>318</v>
+        <v>428</v>
+      </c>
+      <c r="H80" s="5" t="s">
+        <v>429</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="21">
@@ -7040,6 +7163,9 @@
       <c r="E83" s="5" t="s">
         <v>269</v>
       </c>
+      <c r="F83">
+        <v>3</v>
+      </c>
     </row>
     <row r="84" spans="1:8" ht="21">
       <c r="A84">
@@ -7061,7 +7187,7 @@
         <v>3</v>
       </c>
       <c r="H84" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="21">
@@ -7124,7 +7250,7 @@
         <v>3</v>
       </c>
       <c r="H87" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="21">
@@ -7147,7 +7273,7 @@
         <v>1</v>
       </c>
       <c r="H88" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="21">
@@ -7189,6 +7315,9 @@
       <c r="F90">
         <v>2</v>
       </c>
+      <c r="G90">
+        <v>2.2999999999999998</v>
+      </c>
     </row>
     <row r="91" spans="1:8" ht="21">
       <c r="A91">
@@ -7210,7 +7339,7 @@
         <v>1</v>
       </c>
       <c r="H91" s="5" t="s">
-        <v>329</v>
+        <v>430</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="21">

</xml_diff>

<commit_message>
add function classifying with llama 2 change prompts for auto annotation
</commit_message>
<xml_diff>
--- a/annotation_tool/annotation_template.xlsx
+++ b/annotation_tool/annotation_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/heste/workspace/sn-caption/annotation_tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC213EB-103A-F94C-9B0A-F02FED668E5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D947A248-97CB-344A-80B5-91247A2CD87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31180" yWindow="4740" windowWidth="25600" windowHeight="14140" activeTab="3" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
+    <workbookView xWindow="4920" yWindow="-28300" windowWidth="25600" windowHeight="14160" activeTab="3" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
   </bookViews>
   <sheets>
     <sheet name="テンプレート_seed42" sheetId="4" r:id="rId1"/>
@@ -106,7 +106,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="439">
   <si>
     <t>id</t>
   </si>
@@ -1545,6 +1545,10 @@
     <rPh sb="3" eb="5">
       <t xml:space="preserve">ジョウホウ </t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>You can definitely run up to Ludwig, who shows weaknesses more often in the game, the Russian goalkeeper.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -7677,7 +7681,7 @@
         <v>222</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>223</v>
+        <v>438</v>
       </c>
       <c r="F2" t="b">
         <f>G2=2</f>
@@ -7714,7 +7718,7 @@
         <v>3</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="21">
@@ -8251,13 +8255,10 @@
       </c>
       <c r="F25" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>2</v>
-      </c>
-      <c r="H25">
-        <v>1.1000000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="21">
@@ -9040,10 +9041,13 @@
       </c>
       <c r="F57" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G57">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="H57">
+        <v>2.2999999999999998</v>
       </c>
       <c r="I57" s="5" t="s">
         <v>427</v>
@@ -9196,13 +9200,10 @@
       </c>
       <c r="F63" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G63">
-        <v>2</v>
-      </c>
-      <c r="H63">
-        <v>1.1000000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="42">

</xml_diff>

<commit_message>
add script for all comment annotation
</commit_message>
<xml_diff>
--- a/annotation_tool/annotation_template.xlsx
+++ b/annotation_tool/annotation_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/heste/workspace/sn-caption/annotation_tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D947A248-97CB-344A-80B5-91247A2CD87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11EE68CA-F914-A04F-B909-C9E43CE926AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4920" yWindow="-28300" windowWidth="25600" windowHeight="14160" activeTab="3" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="3" xr2:uid="{89A04599-6038-9D4E-8F37-84B4D23DB047}"/>
   </bookViews>
   <sheets>
     <sheet name="テンプレート_seed42" sheetId="4" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <definedName name="denoised_1_tokenized_224p_annotation" localSheetId="0">テンプレート_seed42!$A$1:$H$101</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -106,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="440">
   <si>
     <t>id</t>
   </si>
@@ -1549,6 +1550,10 @@
   </si>
   <si>
     <t>You can definitely run up to Ludwig, who shows weaknesses more often in the game, the Russian goalkeeper.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>He's been taken under the wing by Victor Fernandez but he's going to be slightly off the pace whatever and you're going up against arguably the most potent strike force in all of the Liga if not Europe.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -7834,7 +7839,7 @@
         <v>234</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>235</v>
+        <v>439</v>
       </c>
       <c r="F8" t="b">
         <f>G8=2</f>

</xml_diff>